<commit_message>
Cập nhật README, CLAUDE.md, bảng dữ liệu v0.3 và bảng từ ngoại lai
</commit_message>
<xml_diff>
--- a/asr_tts_o_to_handoff/data/du_lieu_asr_tts_o_to_v0.3.xlsx
+++ b/asr_tts_o_to_handoff/data/du_lieu_asr_tts_o_to_v0.3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder (2)\asr_tts_o_to_handoff\asr_tts_o_to_handoff\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790A2418-5D3D-47C6-B627-01EAB9CC1CCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE6EE99E-5B14-49D7-B4EC-75328DE6F9E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tong_quan" sheetId="1" r:id="rId1"/>
@@ -29,6 +29,7 @@
     <sheet name="Tai_lieu" sheetId="14" r:id="rId14"/>
     <sheet name="Tu_dia_phuong" sheetId="15" r:id="rId15"/>
     <sheet name="Tu_vung" sheetId="16" r:id="rId16"/>
+    <sheet name="Sheet1" sheetId="17" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Mau_cau!$A$3:$R$82</definedName>
@@ -6358,7 +6359,7 @@
       <c r="A7" s="13" t="s">
         <v>644</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="42" t="s">
         <v>1276</v>
       </c>
       <c r="C7" s="14" t="s">
@@ -6748,7 +6749,7 @@
       <c r="A14" s="13" t="s">
         <v>1326</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="42" t="s">
         <v>1327</v>
       </c>
       <c r="C14" s="14" t="s">
@@ -6972,7 +6973,7 @@
       <c r="A18" s="13" t="s">
         <v>1354</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="42" t="s">
         <v>1355</v>
       </c>
       <c r="C18" s="14" t="s">
@@ -9621,6 +9622,15 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0D1F6CC-5B36-41C0-B120-65D9BE032FB2}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K8"/>
@@ -20002,7 +20012,7 @@
         <v>2</v>
       </c>
       <c r="P68" s="14" t="str">
-        <f t="shared" ref="P68:P99" si="5">IF(O68&lt;=3,"Rất ngắn (≤3)",IF(O68&lt;=8,"Ngắn (4–8)","Thường (&gt;8)"))</f>
+        <f t="shared" ref="P68:P82" si="5">IF(O68&lt;=3,"Rất ngắn (≤3)",IF(O68&lt;=8,"Ngắn (4–8)","Thường (&gt;8)"))</f>
         <v>Rất ngắn (≤3)</v>
       </c>
       <c r="Q68" s="13">

</xml_diff>